<commit_message>
Restore logging test report worksheet
</commit_message>
<xml_diff>
--- a/workshop/Workshop_Template_70BG.xlsx
+++ b/workshop/Workshop_Template_70BG.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R7e7485daea6c44e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="2" r:id="Red76be7f9bfa43bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="log" sheetId="3" r:id="R44aab2c583874918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="4" r:id="Ree565ece8c2a4f73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" r:id="R43019daaedb64f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listen" sheetId="2" r:id="R60d4a818d68842fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="log" sheetId="3" r:id="R5a166bf27eb342de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="log_Testbericht" sheetId="4" r:id="R61294060ea7f45a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -54,8 +54,12 @@
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="15"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:sz val="14"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -88,7 +92,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF17365D"/>
+        <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -140,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -207,19 +211,20 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -8011,63 +8016,214 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="95" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="50" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="32" t="str">
-        <x:v>Workshop template – Hinweise</x:v>
-      </x:c>
-      <x:c r="B1" s="32"/>
-      <x:c r="C1" s="32"/>
-      <x:c r="D1" s="32"/>
-      <x:c r="E1" s="32"/>
-      <x:c r="F1" s="32"/>
-    </x:row>
-    <x:row r="3" ht="45" customHeight="1">
-      <x:c r="A3" s="34" t="str">
-        <x:v>1. BG-Daten eintragen</x:v>
-      </x:c>
-      <x:c r="B3" s="35" t="str">
-        <x:v>In Template die Spalten A–E befüllen und in F je Zeile den Screenshot einfügen. H–L bleiben für die Teilnehmenden leer.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="45" customHeight="1">
-      <x:c r="A4" s="34" t="str">
-        <x:v>2. Dropdowns</x:v>
-      </x:c>
-      <x:c r="B4" s="35" t="str">
-        <x:v>H und J verwenden dieselben sieben Baugruppen-Klassen. I verwendet vier Konfidenzstufen. K und L sind Freitext.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="45" customHeight="1">
-      <x:c r="A5" s="34" t="str">
-        <x:v>3. Zeitstempel</x:v>
-      </x:c>
-      <x:c r="B5" s="35" t="str">
-        <x:v>Das Blatt log nutzt selbstreferenzierende Formeln. In Excel muss Datei &gt; Optionen &gt; Formeln &gt; Iterative Berechnung aktivieren eingeschaltet sein; maximale Iterationen: 1.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="45" customHeight="1">
-      <x:c r="A6" s="34" t="str">
-        <x:v>4. Verwendung</x:v>
-      </x:c>
-      <x:c r="B6" s="35" t="str">
-        <x:v>Pro Teilnehmendem eine eigene Dateikopie verwenden. Der Log dokumentiert Felder, aber keinen Bearbeiternamen.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="45" customHeight="1">
-      <x:c r="A7" s="34" t="str">
-        <x:v>5. Achtung</x:v>
-      </x:c>
-      <x:c r="B7" s="35" t="str">
-        <x:v>Keine Zeilen in Template oder log löschen bzw. einfügen. Nur die vorgesehenen Zellen ausfüllen oder Inhalte ersetzen.</x:v>
-      </x:c>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="31" t="str">
+        <x:v>Testbericht Logging-Tool (Blatt 'log')</x:v>
+      </x:c>
+      <x:c r="B1" s="31"/>
+      <x:c r="C1" s="31"/>
+      <x:c r="D1" s="31"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="32" t="str">
+        <x:v>Nr</x:v>
+      </x:c>
+      <x:c r="B2" s="32" t="str">
+        <x:v>Testfall</x:v>
+      </x:c>
+      <x:c r="C2" s="32" t="str">
+        <x:v>Befund (vorher)</x:v>
+      </x:c>
+      <x:c r="D2" s="32" t="str">
+        <x:v>Status / Maßnahme (nachher)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="33" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B3" s="33" t="str">
+        <x:v>Eintrag setzen (z. B. Klasse wählen)</x:v>
+      </x:c>
+      <x:c r="C3" s="33" t="str">
+        <x:v>TS1 wird korrekt gestempelt</x:v>
+      </x:c>
+      <x:c r="D3" s="33" t="str">
+        <x:v>OK – unverändert übernommen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>Feld leeren</x:v>
+      </x:c>
+      <x:c r="C4" s="33" t="str">
+        <x:v>Geleert-Zeitstempel korrekt</x:v>
+      </x:c>
+      <x:c r="D4" s="33" t="str">
+        <x:v>OK – unverändert übernommen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="33" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B5" s="33" t="str">
+        <x:v>Wiedereintrag nach Leeren</x:v>
+      </x:c>
+      <x:c r="C5" s="33" t="str">
+        <x:v>TS2 korrekt</x:v>
+      </x:c>
+      <x:c r="D5" s="33" t="str">
+        <x:v>OK – unverändert übernommen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="33" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="str">
+        <x:v>3. und weitere Änderungszyklen</x:v>
+      </x:c>
+      <x:c r="C6" s="33" t="str">
+        <x:v>Nicht erfasst – alle Änderungen nach TS2 unsichtbar</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="str">
+        <x:v>Erfasst über Erster Wert, Aktuell und Änderungsverlauf je Feld</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="33" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="33" t="str">
+        <x:v>Wert direkt überschreiben (ohne Leeren)</x:v>
+      </x:c>
+      <x:c r="C7" s="33" t="str">
+        <x:v>Kein Log-Eintrag – Änderung unsichtbar</x:v>
+      </x:c>
+      <x:c r="D7" s="33" t="str">
+        <x:v>Erfasst über Aktuell je Feld</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="33" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="33" t="str">
+        <x:v>Fehlerwert in Quellzelle (z. B. #NV)</x:v>
+      </x:c>
+      <x:c r="C8" s="33" t="str">
+        <x:v>Fehler schrieb sich dauerhaft ins Log</x:v>
+      </x:c>
+      <x:c r="D8" s="33" t="str">
+        <x:v>Fehlerbehandlung in den Log-Formeln</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="33" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B9" s="33" t="str">
+        <x:v>Zeile im Template löschen/einfügen</x:v>
+      </x:c>
+      <x:c r="C9" s="33" t="str">
+        <x:v>Dauerhafte #BEZUG!-Fehler</x:v>
+      </x:c>
+      <x:c r="D9" s="33" t="str">
+        <x:v>Keine Zeilen in Template oder log löschen bzw. einfügen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="33" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B10" s="33" t="str">
+        <x:v>Objekte ab Zeile 21</x:v>
+      </x:c>
+      <x:c r="C10" s="33" t="str">
+        <x:v>Nur ein Teil der Zeilen abgedeckt</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str">
+        <x:v>Log ist für 70 Workshop-BGs vorbereitet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="33" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B11" s="33" t="str">
+        <x:v>Nur Leerzeichen eingeben</x:v>
+      </x:c>
+      <x:c r="C11" s="33" t="str">
+        <x:v>Zählte als gültiger Eintrag</x:v>
+      </x:c>
+      <x:c r="D11" s="33" t="str">
+        <x:v>TRIM: Leerzeichen gelten als leer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="33" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B12" s="33" t="str">
+        <x:v>Zahl 0 als Eingabe</x:v>
+      </x:c>
+      <x:c r="C12" s="33" t="str">
+        <x:v>Korrekt geloggt</x:v>
+      </x:c>
+      <x:c r="D12" s="33" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="33" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B13" s="33" t="str">
+        <x:v>Reparatur/Formeltausch auf gestempelter Zelle</x:v>
+      </x:c>
+      <x:c r="C13" s="33" t="str">
+        <x:v>Original-Zeitstempel ging verloren</x:v>
+      </x:c>
+      <x:c r="D13" s="33" t="str">
+        <x:v>Stempel nachträglich nicht manuell überschreiben</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B14" s="33" t="str">
+        <x:v>Voraussetzung: Iterative Berechnung</x:v>
+      </x:c>
+      <x:c r="C14" s="33" t="str">
+        <x:v>Muss aktiviert sein</x:v>
+      </x:c>
+      <x:c r="D14" s="33" t="str">
+        <x:v>Datei &gt; Optionen &gt; Formeln: aktiv, maximale Iterationen 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="36" t="str">
+        <x:v>Hinweise: Der Log erfasst Zeitpunkte pro Feld, keine Benutzer. Bei mehreren Bearbeitern ggf. Spalte 'Teilnehmer' im Template ergänzen.</x:v>
+      </x:c>
+      <x:c r="B16" s="36"/>
+      <x:c r="C16" s="36"/>
+      <x:c r="D16" s="36"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A16:D16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>